<commit_message>
Update Kenya crop classification and mark all countries (except GHA) as active
- Updated crops.json and crops_from_excel.json with new KEN classification hierarchy
- Updated List_of_crops_update_all_3.xlsx source file
- README: MOZ, ZMB, KEN now marked as Active (6/7 countries live)
- README: Version bumped to 1.3.0, updated project status and changelog

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/List_of_crops_update_all_3.xlsx
+++ b/List_of_crops_update_all_3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\antigravity\Land cover\github\Land-cover-validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5359F5E2-0514-465E-97EF-D685B86B6202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BAE4D40-CA25-4100-A52A-EF5E5FC49B12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="770" yWindow="4280" windowWidth="23230" windowHeight="10180" xr2:uid="{ADA269A6-2ED3-4A77-8230-6F13C182E555}"/>
+    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" activeTab="4" xr2:uid="{ADA269A6-2ED3-4A77-8230-6F13C182E555}"/>
   </bookViews>
   <sheets>
     <sheet name="Crop_list_HND" sheetId="8" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1494" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1524" uniqueCount="291">
   <si>
     <t>Level_1</t>
   </si>
@@ -892,13 +892,40 @@
   </si>
   <si>
     <t>Artificial waterbody</t>
+  </si>
+  <si>
+    <t>Dryland rice</t>
+  </si>
+  <si>
+    <t>Monkeynuts</t>
+  </si>
+  <si>
+    <t>Pineapples</t>
+  </si>
+  <si>
+    <t>Greenhouses</t>
+  </si>
+  <si>
+    <t>Sisal</t>
+  </si>
+  <si>
+    <t>Snow</t>
+  </si>
+  <si>
+    <t>Salt pans</t>
+  </si>
+  <si>
+    <t>Ocean</t>
+  </si>
+  <si>
+    <t>Vegetated Wetlands</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -968,8 +995,15 @@
       <color rgb="FF000000"/>
       <name val="Aptos"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1042,8 +1076,14 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1147,11 +1187,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1194,6 +1245,18 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4381,7 +4444,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F421573-7F45-40AE-9E4F-984A0D6DDEFC}">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C98"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33.26953125" customWidth="1"/>
@@ -4404,10 +4467,10 @@
       <c r="A2" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="32" t="s">
         <v>155</v>
       </c>
     </row>
@@ -4415,10 +4478,10 @@
       <c r="A3" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="32" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4426,10 +4489,10 @@
       <c r="A4" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="32" t="s">
         <v>121</v>
       </c>
     </row>
@@ -4437,10 +4500,10 @@
       <c r="A5" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="32" t="s">
         <v>156</v>
       </c>
     </row>
@@ -4448,10 +4511,10 @@
       <c r="A6" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="32" t="s">
         <v>123</v>
       </c>
     </row>
@@ -4459,10 +4522,10 @@
       <c r="A7" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="32" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4470,10 +4533,10 @@
       <c r="A8" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="B8" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" s="32" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4481,10 +4544,10 @@
       <c r="A9" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="32" t="s">
         <v>157</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="32" t="s">
         <v>157</v>
       </c>
     </row>
@@ -4492,10 +4555,10 @@
       <c r="A10" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="32" t="s">
         <v>157</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="32" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4503,10 +4566,10 @@
       <c r="A11" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="32" t="s">
         <v>158</v>
       </c>
     </row>
@@ -4514,10 +4577,10 @@
       <c r="A12" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="32" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4525,10 +4588,10 @@
       <c r="A13" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="B13" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="32" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4536,10 +4599,10 @@
       <c r="A14" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="32" t="s">
         <v>159</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="32" t="s">
         <v>159</v>
       </c>
     </row>
@@ -4547,10 +4610,10 @@
       <c r="A15" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="32" t="s">
         <v>124</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="32" t="s">
         <v>124</v>
       </c>
     </row>
@@ -4558,10 +4621,10 @@
       <c r="A16" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="32" t="s">
         <v>125</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="32" t="s">
         <v>125</v>
       </c>
     </row>
@@ -4569,10 +4632,10 @@
       <c r="A17" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="B17" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" s="32" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4580,7 +4643,7 @@
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C18" s="3" t="s">
@@ -4591,7 +4654,7 @@
       <c r="A19" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C19" s="3" t="s">
@@ -4602,7 +4665,7 @@
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C20" s="3" t="s">
@@ -4613,7 +4676,7 @@
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C21" s="3" t="s">
@@ -4624,7 +4687,7 @@
       <c r="A22" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C22" s="3" t="s">
@@ -4635,7 +4698,7 @@
       <c r="A23" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C23" s="3" t="s">
@@ -4646,7 +4709,7 @@
       <c r="A24" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C24" s="3" t="s">
@@ -4657,7 +4720,7 @@
       <c r="A25" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C25" s="3" t="s">
@@ -4668,7 +4731,7 @@
       <c r="A26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C26" s="3" t="s">
@@ -4679,7 +4742,7 @@
       <c r="A27" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C27" s="3" t="s">
@@ -4690,7 +4753,7 @@
       <c r="A28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C28" s="3" t="s">
@@ -4701,7 +4764,7 @@
       <c r="A29" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C29" s="3" t="s">
@@ -4712,7 +4775,7 @@
       <c r="A30" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C30" s="3" t="s">
@@ -4723,7 +4786,7 @@
       <c r="A31" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="32" t="s">
         <v>92</v>
       </c>
       <c r="C31" s="3" t="s">
@@ -4734,260 +4797,260 @@
       <c r="A32" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="C32" s="24" t="s">
+      <c r="C32" s="32" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A33" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>90</v>
+      <c r="A33" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" s="34" t="s">
+        <v>178</v>
+      </c>
+      <c r="C33" s="34" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="32" t="s">
         <v>87</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>166</v>
+        <v>90</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="32" t="s">
         <v>87</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>88</v>
+        <v>166</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A36" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B36" s="2" t="s">
+      <c r="A36" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="C36" s="3" t="s">
-        <v>91</v>
+      <c r="C36" s="35" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A37" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="32" t="s">
         <v>87</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A38" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="32" t="s">
         <v>87</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>136</v>
+        <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A39" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="C39" s="24" t="s">
-        <v>79</v>
+      <c r="C39" s="3" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>106</v>
+      <c r="B40" s="32" t="s">
+        <v>87</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>167</v>
+        <v>136</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A41" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>138</v>
+      <c r="B41" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="C41" s="32" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A42" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="32" t="s">
         <v>106</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A43" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="32" t="s">
         <v>106</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>169</v>
+        <v>138</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A44" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="32" t="s">
         <v>106</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>139</v>
+        <v>168</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A45" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" s="32" t="s">
         <v>106</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>140</v>
+        <v>169</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A46" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="32" t="s">
         <v>106</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A47" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="32" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="24" t="s">
-        <v>79</v>
+      <c r="C47" s="3" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A48" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>170</v>
+      <c r="A48" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B48" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="C48" s="35" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>111</v>
+      <c r="B49" s="32" t="s">
+        <v>106</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>171</v>
+        <v>141</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A50" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>112</v>
+      <c r="B50" s="32" t="s">
+        <v>106</v>
+      </c>
+      <c r="C50" s="32" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A51" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A52" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>173</v>
+        <v>112</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A53" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B53" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A54" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A55" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C55" s="3" t="s">
@@ -4998,7 +5061,7 @@
       <c r="A56" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C56" s="3" t="s">
@@ -5009,352 +5072,462 @@
       <c r="A57" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A58" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A59" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B59" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A60" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A61" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A62" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A63" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="B63" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A64" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" s="32" t="s">
         <v>111</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>185</v>
+        <v>152</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A65" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="32" t="s">
         <v>111</v>
       </c>
-      <c r="C65" s="3" t="s">
-        <v>186</v>
+      <c r="C65" s="32" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A66" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>150</v>
+      <c r="A66" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B66" s="34" t="s">
+        <v>284</v>
+      </c>
+      <c r="C66" s="34" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A67" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>152</v>
+      <c r="A67" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B67" s="34" t="s">
+        <v>266</v>
+      </c>
+      <c r="C67" s="34" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A68" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C68" s="24" t="s">
-        <v>79</v>
+      <c r="A68" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B68" s="34" t="s">
+        <v>266</v>
+      </c>
+      <c r="C68" s="34" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A69" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>188</v>
+      <c r="A69" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B69" s="34" t="s">
+        <v>266</v>
+      </c>
+      <c r="C69" s="34" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A70" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>190</v>
+      <c r="A70" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B70" s="34" t="s">
+        <v>266</v>
+      </c>
+      <c r="C70" s="34" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A71" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C71" s="3" t="s">
-        <v>191</v>
+      <c r="A71" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B71" s="34" t="s">
+        <v>266</v>
+      </c>
+      <c r="C71" s="34" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A72" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" ht="32" x14ac:dyDescent="0.4">
-      <c r="A73" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>193</v>
+      <c r="A72" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B72" s="34" t="s">
+        <v>285</v>
+      </c>
+      <c r="C72" s="34" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+      <c r="A73" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B73" s="34" t="s">
+        <v>286</v>
+      </c>
+      <c r="C73" s="34" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A74" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>194</v>
+      <c r="A74" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B74" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="C74" s="34" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A75" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B75" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>79</v>
+      <c r="B75" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A76" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>195</v>
+        <v>153</v>
+      </c>
+      <c r="B76" s="32" t="s">
+        <v>189</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A77" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>196</v>
+        <v>153</v>
+      </c>
+      <c r="B77" s="32" t="s">
+        <v>189</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A78" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+        <v>153</v>
+      </c>
+      <c r="B78" s="32" t="s">
+        <v>189</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" ht="32" x14ac:dyDescent="0.4">
       <c r="A79" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>198</v>
+        <v>153</v>
+      </c>
+      <c r="B79" s="32" t="s">
+        <v>189</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A80" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>79</v>
+        <v>153</v>
+      </c>
+      <c r="B80" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="C80" s="32" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A81" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>200</v>
+        <v>153</v>
+      </c>
+      <c r="B81" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="C81" s="32" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A82" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>79</v>
+        <v>154</v>
+      </c>
+      <c r="B82" s="32" t="s">
+        <v>195</v>
+      </c>
+      <c r="C82" s="32" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A83" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>201</v>
+        <v>154</v>
+      </c>
+      <c r="B83" s="32" t="s">
+        <v>196</v>
+      </c>
+      <c r="C83" s="32" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="84" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A84" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>202</v>
+        <v>154</v>
+      </c>
+      <c r="B84" s="32" t="s">
+        <v>197</v>
+      </c>
+      <c r="C84" s="32" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A85" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>203</v>
+        <v>154</v>
+      </c>
+      <c r="B85" s="32" t="s">
+        <v>198</v>
+      </c>
+      <c r="C85" s="32" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A86" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>204</v>
+      <c r="A86" s="33" t="s">
+        <v>154</v>
+      </c>
+      <c r="B86" s="34" t="s">
+        <v>287</v>
+      </c>
+      <c r="C86" s="34" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="16" x14ac:dyDescent="0.4">
-      <c r="A87" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>205</v>
+      <c r="A87" s="33" t="s">
+        <v>154</v>
+      </c>
+      <c r="B87" s="34" t="s">
+        <v>288</v>
+      </c>
+      <c r="C87" s="34" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A88" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B88" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="C88" s="32" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+      <c r="A89" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B89" s="32" t="s">
+        <v>200</v>
+      </c>
+      <c r="C89" s="32" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+      <c r="A90" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B90" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="C90" s="32" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+      <c r="A91" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B88" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="C88" s="24" t="s">
-        <v>79</v>
+      <c r="B91" s="32" t="s">
+        <v>63</v>
+      </c>
+      <c r="C91" s="32" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+      <c r="A92" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="B92" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="C92" s="34" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+      <c r="A93" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B93" s="32" t="s">
+        <v>63</v>
+      </c>
+      <c r="C93" s="32" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+      <c r="A94" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B94" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="C94" s="32" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+      <c r="A95" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B95" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="C95" s="32" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+      <c r="A96" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B96" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="C96" s="32" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+      <c r="A97" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B97" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="C97" s="32" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" ht="16" x14ac:dyDescent="0.4">
+      <c r="A98" s="36" t="s">
+        <v>290</v>
+      </c>
+      <c r="B98" s="37" t="s">
+        <v>290</v>
+      </c>
+      <c r="C98" s="37" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>